<commit_message>
Update supplementary table numbering
This updates the numbers of the supplementary tables (e.g. S1, S2 etc) to match the order their citations appear in the text
</commit_message>
<xml_diff>
--- a/Supplementary Information/S1 Cohort Summary.xlsx
+++ b/Supplementary Information/S1 Cohort Summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devin\Desktop\paper\claude\final resubmission\Supplementary Information\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devin\Desktop\rrms\Supplementary Information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0EED87-90E1-429B-B936-74511F73A757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DFAEF3C-600C-4E83-8F60-F8742D1AD8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="368" yWindow="368" windowWidth="26182" windowHeight="14407" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cohort" sheetId="1" r:id="rId1"/>
@@ -353,7 +353,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,6 +376,12 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -425,7 +431,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -442,6 +448,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -745,13 +752,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="52" customWidth="1"/>
-    <col min="2" max="6" width="20" customWidth="1"/>
+    <col min="1" max="1" width="52" style="6" customWidth="1"/>
+    <col min="2" max="6" width="20" style="6" customWidth="1"/>
+    <col min="7" max="16384" width="9.06640625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>74</v>
@@ -769,7 +777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -799,7 +807,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -849,7 +857,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -899,7 +907,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
@@ -1069,7 +1077,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>40</v>
       </c>
@@ -1139,7 +1147,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>49</v>
       </c>
@@ -1229,7 +1237,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>55</v>
       </c>
@@ -1479,7 +1487,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>71</v>
       </c>

</xml_diff>